<commit_message>
Thêm báo cáo Word, slide thuyết trình và cập nhật báo cáo theo công thức 5D
- Báo cáo LaTeX (Springer, IEEE): công thức S theo khung 5D của BOD 26-04, mục BOD 26-04, tình huống điển hình, thang điểm khuyến nghị, rà soát câu từ và nguồn
- Báo cáo Word theo mẫu bìa HUST (ReportWord/BaoCao_Nhom14.docx) và bản PDF của hai báo cáo LaTeX
- Slide thuyết trình 20 trang theo theme HUST, có ghi chú thuyết trình (Slide/)
- Chạy lại notebook, cập nhật kết quả và Y_TUONG.md

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Thu_Kha_Thi/notebooks/ket_qua_bo_sung/bang_bo_sung.xlsx
+++ b/Thu_Kha_Thi/notebooks/ket_qua_bo_sung/bang_bo_sung.xlsx
@@ -1,17 +1,17 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="A1 Theo khoi luong va" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="A2 Mo phong" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="A3 Truoc KEV theo tuoi" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="A4 Nhom khan cap" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="A5 Pham vi kiem thu" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="A1 Theo khoi luong va" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="A2 Mo phong" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="A3 Truoc KEV theo tuoi" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="A4 Nhom khan cap" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="A5 Pham vi kiem thu" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>

</xml_diff>